<commit_message>
Adding more entries and corrections to the files based on testing in-game. Removed quests from Nazgrel because they were fixed into the data query and now are duplicated.
</commit_message>
<xml_diff>
--- a/corrections/corrections.xlsx
+++ b/corrections/corrections.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Desktop\wow_vo_webui\corrections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF6A1CE-99B8-4F11-8281-D8418C429E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784CA0AC-AC1B-4D17-8648-2FB606D3C093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="quest" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="143">
   <si>
     <t>source</t>
   </si>
@@ -491,6 +491,31 @@
     <t>In my travels across this world I have made several interesting discoveries. For instance, did you know that with the proper amount of encouragement one can extract all the truths that a man dares hide? As luck would have it, I happen to have some encouragement on hand.
 These are my persuaders; Equip them and take to the field, death knight; Apply the pointy ends to the soldiers of New Avalon; Discover the truth about this "Crimson Dawn."</t>
   </si>
+  <si>
+    <t>Your beliefs are alien to us, heathen. Ancient Zandalar were once branded as heretics. This was when the Gurubashi Empire was strong. Heathens dared to challenge the priest of Hakkar. Heathens then were hunted and killed as vermin. Those heathens never wavered in their fight against the Blood God. We honor the price they paid. They are the freethinkers.
+Destroy the minions of Hakkar in Zul'Gurub; Bring me the Paragons of Power I seek; Success will be greatly rewarded.
+Go.</t>
+  </si>
+  <si>
+    <t>pirate</t>
+  </si>
+  <si>
+    <t>What's this? With the four sigils brought together, they have formed together to create one sigil. There can be no doubt that this will be able to break the wardings placed upon Trollbane's tomb.
+Trollbane's remains are entombed in the Sanctum behind the chapel in Stromgarde; Retrieve Trol'kalar.</t>
+  </si>
+  <si>
+    <t>The light slowly fades; the sword Trol'kalar, held within a stone sheath has been released.</t>
+  </si>
+  <si>
+    <t>Well done, adventurer; That's one less forge camp we'll need to worry about. It'll take the Legion a while to get that facility back up and running. You've just bought us the one thing we'd run out of; time.</t>
+  </si>
+  <si>
+    <t>You are an honor to us, But now we must strike before the Legion recovers! To the north of Thrallmar lies Invasion Point Annihilator; It houses a warp-portal through which the Legion draws its reinforcements.
+You must overload that portal - and blast it back to the abyss it came from. The portal's activation key will be held by the Point's commander - Warbringer Arix'Amal. Slay him. Take the key. Use it on the portal and do what must be done. May the warchief's blessings be with you.</t>
+  </si>
+  <si>
+    <t>Greetings, adventurer; I've deciphered the Legion missive and uncovered the demons' strategic plans for this Peninsula. Apparently, there is a large group of hellish terrorfiends gathering near the Pools of Aggonar in the west. We cannot allow such a force to go unchallenged. You must go there and decimate their cursed numbers.</t>
+  </si>
 </sst>
 </file>
 
@@ -879,7 +904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56545B79-22C0-4057-A076-1E697524330B}">
-  <dimension ref="A1:F1104"/>
+  <dimension ref="A1:F1110"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -9860,8 +9885,74 @@
       <c r="B1104">
         <v>12720</v>
       </c>
-      <c r="D1104" s="1" t="s">
+      <c r="D1104" t="s">
         <v>135</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1105" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1105">
+        <v>8054</v>
+      </c>
+      <c r="D1105" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1106" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1106">
+        <v>645</v>
+      </c>
+      <c r="D1106" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1107" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1107">
+        <v>646</v>
+      </c>
+      <c r="D1107" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1108" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1108">
+        <v>10390</v>
+      </c>
+      <c r="D1108" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1109" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1109">
+        <v>10392</v>
+      </c>
+      <c r="D1109" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1110" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1110">
+        <v>10389</v>
+      </c>
+      <c r="D1110" s="1" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -9880,7 +9971,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D60A7C4-82C4-4AAF-A00A-127D625F91A3}">
-  <dimension ref="A1:H729"/>
+  <dimension ref="A1:H734"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -12575,7 +12666,7 @@
         <v>17877</v>
       </c>
       <c r="E308" t="s">
-        <v>41</v>
+        <v>134</v>
       </c>
     </row>
     <row r="309" spans="1:5" x14ac:dyDescent="0.25">
@@ -13295,7 +13386,7 @@
         <v>2610</v>
       </c>
       <c r="E398" t="s">
-        <v>33</v>
+        <v>137</v>
       </c>
     </row>
     <row r="399" spans="1:5" x14ac:dyDescent="0.25">
@@ -15959,6 +16050,46 @@
       </c>
       <c r="E729" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="730" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A730">
+        <v>23995</v>
+      </c>
+      <c r="B730">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="731" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A731">
+        <v>29590</v>
+      </c>
+      <c r="B731">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="732" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A732">
+        <v>28552</v>
+      </c>
+      <c r="B732">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="733" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A733">
+        <v>24975</v>
+      </c>
+      <c r="B733">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="734" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A734">
+        <v>18063</v>
+      </c>
+      <c r="E734" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>